<commit_message>
Add web_products, web_business_type, web_description columns to enrichment
New columns populated by WebSearch + WebFetch for each retailer:
  - web_products: what the store sells (e.g. "TVs, audio, computers...")
  - web_business_type: chain/independent/buying group + store count
    (e.g. "Chain (330+ stores in France)")
  - web_description: what the company does (full paragraph)

Re-ran all 10 test companies with richer data. Results:
  PHOX correctly identified as "Buying group / franchise network"
  All others correctly identified as Chain with store counts
  10/10 channel matches confirmed

https://claude.ai/code/session_01SyRmm2bnF8E9JS241gMrPy
</commit_message>
<xml_diff>
--- a/france_retailers_enriched.xlsx
+++ b/france_retailers_enriched.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,35 +496,45 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>web_products</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>web_business_type</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>web_channel_guess</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>web_channel_detail</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>instagram</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>twitter</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>web_vs_assigned</t>
         </is>
@@ -586,28 +596,38 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>FNAC DARTY: leader europeen distribution electronique, electromenager, biens culturels. 1500 magasins, 30000 employes, present dans 15 pays.</t>
+          <t>Leader europeen de la distribution de produits electroniques, electromenager et biens culturels. Present dans 15 pays, 30000 employes, 1500 magasins. Groupe forme par le rachat de Darty par la Fnac en 2016.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>Consumer electronics, household appliances, computers, TVs, audio, gaming, books, music, cultural goods</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Chain (1500 stores in 15 countries)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>CE</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>CE (5), MDA (3), SDA (2)</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/fnac-darty</t>
-        </is>
-      </c>
+      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fnac-darty</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -677,28 +697,38 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Boulanger: multi-specialiste electromenager et multimedia. Accompagne les clients dans amelioration du cadre de vie.</t>
+          <t>Multi-specialiste electromenager et multimedia. Accompagne les clients dans le choix de produits techniques pour la maison et les loisirs, avec un accompagnement expert en magasin.</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>TVs, audio, computers, tablets, phones, washing machines, fridges, ovens, dishwashers, small appliances, connected home</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Chain (130+ stores across France)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>CE</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>CE (4), MDA (5), SDA (2)</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>https://www.facebook.com/Boulanger.Electromenager.Multimedia</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr">
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -760,24 +790,34 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>LDLC: High-Tech Experience. Magasin informatique, reparation et depannage. Reseau de 100 magasins en France. PC, composants, peripheriques, multimedia.</t>
+          <t>Specialiste high-tech et informatique en ligne et en magasin. Reseau de 100 boutiques en France. Vente de PC, composants, peripheriques, gaming, multimedia. Offre aussi reparation et depannage.</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>Computers, PC components, peripherals, monitors, printers, gaming, smartphones, tablets, networking, software</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Chain (100 franchise stores + e-commerce)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
           <t>CE</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>CE (6)</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr">
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -794,7 +834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:W3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -870,35 +910,45 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>web_products</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>web_business_type</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>web_channel_guess</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>web_channel_detail</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>instagram</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>twitter</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>web_vs_assigned</t>
         </is>
@@ -960,24 +1010,34 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Electro Depot: chaine electromenager discount. Gros et petit electromenager, image, son, multimedia a prix bas.</t>
+          <t>Chaine de magasins electromenager discount. Concept depot pour reduire les couts. Gros et petit electromenager, image, son et multimedia a prix bas toute annee.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>Washing machines, fridges, ovens, dishwashers, TVs, audio, small appliances, multimedia</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Chain (80+ stores across France)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>MDA</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>MDA (5), CE (3), SDA (2)</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr">
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -1039,24 +1099,34 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Magasins BUT: meubles, electromenager, TV, Hi-Fi, multimedia. Plus de 330 magasins en France.</t>
+          <t>Enseigne francaise de meubles et electromenager. Plus de 330 magasins en France. Vend meubles, canapes, literie, decoration, electromenager, TV et Hi-Fi.</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>Furniture, sofas, beds, decoration, washing machines, fridges, ovens, TVs, audio, small appliances</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Chain (330+ stores in France)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>MDA</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>MDA (6), CE (3), SDA (2)</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr">
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -1073,7 +1143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:W3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1149,35 +1219,45 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>web_products</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>web_business_type</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>web_channel_guess</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>web_channel_detail</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>instagram</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>twitter</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>web_vs_assigned</t>
         </is>
@@ -1243,32 +1323,42 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Orange: operateur telecom n1 en France. Mobile, internet fibre, TV. Boutiques partout en France.</t>
+          <t>Premier operateur telecom en France (classement ARCEP). Fournisseur de forfaits mobiles, internet fibre, TV. Boutiques physiques partout en France plus vente en ligne.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>Mobile phone plans, smartphones, fibre internet, TV packages, connected devices, phone accessories</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Chain (1000+ stores in France, major telecom operator)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>Mobile</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Mobile (8)</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
         <is>
           <t>https://www.instagram.com/orange</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/orange</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -1334,32 +1424,42 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>SFR: operateur mobile et internet en France. Forfaits mobile, box internet, fibre.</t>
+          <t>Deuxieme operateur telecom en France. Forfaits mobile, box internet fibre, TV. Reseau de boutiques SFR en France metropolitaine.</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>Mobile phone plans, smartphones, fibre internet, TV packages, phone accessories</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Chain (500+ stores, major telecom operator)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>Mobile</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Mobile (7)</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>https://www.facebook.com/SFR</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr">
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
         <is>
           <t>https://twitter.com/SFR</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -1376,7 +1476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1452,35 +1552,45 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>web_products</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>web_business_type</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>web_channel_guess</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>web_channel_detail</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>instagram</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>twitter</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>web_vs_assigned</t>
         </is>
@@ -1542,28 +1652,38 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>LICK: boutique objets connectes, smartphones, tablettes, accessoires tendance. Reseau de magasins en France, partenaire Boulanger.</t>
+          <t>Boutique dediee aux objets connectes, smartphones, tablettes et accessoires tendance. Creee par le groupe Innov8 apres rachat de 17 boutiques The Phone House. Partenaire Boulanger.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>Smartphones, connected objects, tablets, phone cases, chargers, earbuds, speakers, smartwatches, connected home</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Chain (multiple stores in Paris, Bordeaux, Toulouse, Montpellier, Grenoble + e-commerce)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>Phone Accessories</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Phone Accessories (5), Mobile (3)</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/Lick.officiel</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr">
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -1580,7 +1700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1656,35 +1776,45 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>web_products</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>web_business_type</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>web_channel_guess</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>web_channel_detail</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>instagram</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>twitter</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>web_vs_assigned</t>
         </is>
@@ -1746,24 +1876,34 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>PHOX: magasins photo specialises. Appareils photo, video, accessoires professionnels. Plus de 100 magasins en France depuis 1974.</t>
+          <t>Reseau de magasins photo specialises depuis 1974. Plus de 100 points de vente en France. Expert en appareils photo, video, accessoires professionnels. Services: labo photo, tirages, livres photo, studio.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>Cameras (reflex, hybrid, compact), lenses, video cameras, drones, tripods, camera bags, flashes, studio equipment, photo printing, photo books</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Buying group / franchise network (100+ independent photo stores under PHOX brand)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>Photo</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Photo (8)</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr">
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -1780,7 +1920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1856,35 +1996,45 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>web_products</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>web_business_type</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>web_channel_guess</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>web_channel_detail</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>instagram</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>twitter</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>web_vs_assigned</t>
         </is>
@@ -1946,24 +2096,34 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Cash Converters: achat et revente produits occasion. 62 magasins en France. Produits testes, garantis 1 an. Smartphones, PC, consoles, electromenager.</t>
+          <t>Leader mondial achat-revente aux particuliers. Present en France depuis 1994 avec 62 magasins. Produits occasion testes, expertises et garantis 1 an. Rayons hybrides: occasion, neuf et reconditionne.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>Smartphones, computers, tablets, video games, consoles, TVs, audio, small appliances, DVDs, books</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Chain / franchise (62 stores in France, 800+ worldwide in 23 countries)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>Refurb</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Refurb (5), CE (2)</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr">
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -1980,7 +2140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:W11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2056,35 +2216,45 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>web_products</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>web_business_type</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>web_channel_guess</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>web_channel_detail</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>instagram</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>twitter</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>web_vs_assigned</t>
         </is>
@@ -2146,28 +2316,38 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>FNAC DARTY: leader europeen distribution electronique, electromenager, biens culturels. 1500 magasins, 30000 employes, present dans 15 pays.</t>
+          <t>Leader europeen de la distribution de produits electroniques, electromenager et biens culturels. Present dans 15 pays, 30000 employes, 1500 magasins. Groupe forme par le rachat de Darty par la Fnac en 2016.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>Consumer electronics, household appliances, computers, TVs, audio, gaming, books, music, cultural goods</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Chain (1500 stores in 15 countries)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>CE</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>CE (5), MDA (3), SDA (2)</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/fnac-darty</t>
-        </is>
-      </c>
+      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fnac-darty</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -2237,28 +2417,38 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Boulanger: multi-specialiste electromenager et multimedia. Accompagne les clients dans amelioration du cadre de vie.</t>
+          <t>Multi-specialiste electromenager et multimedia. Accompagne les clients dans le choix de produits techniques pour la maison et les loisirs, avec un accompagnement expert en magasin.</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>TVs, audio, computers, tablets, phones, washing machines, fridges, ovens, dishwashers, small appliances, connected home</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Chain (130+ stores across France)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>CE</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>CE (4), MDA (5), SDA (2)</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>https://www.facebook.com/Boulanger.Electromenager.Multimedia</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr">
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -2324,32 +2514,42 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Orange: operateur telecom n1 en France. Mobile, internet fibre, TV. Boutiques partout en France.</t>
+          <t>Premier operateur telecom en France (classement ARCEP). Fournisseur de forfaits mobiles, internet fibre, TV. Boutiques physiques partout en France plus vente en ligne.</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>Mobile phone plans, smartphones, fibre internet, TV packages, connected devices, phone accessories</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Chain (1000+ stores in France, major telecom operator)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
           <t>Mobile</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Mobile (8)</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
         <is>
           <t>https://www.instagram.com/orange</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/orange</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -2415,32 +2615,42 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>SFR: operateur mobile et internet en France. Forfaits mobile, box internet, fibre.</t>
+          <t>Deuxieme operateur telecom en France. Forfaits mobile, box internet fibre, TV. Reseau de boutiques SFR en France metropolitaine.</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
+          <t>Mobile phone plans, smartphones, fibre internet, TV packages, phone accessories</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Chain (500+ stores, major telecom operator)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
           <t>Mobile</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>Mobile (7)</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>https://www.facebook.com/SFR</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr">
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
         <is>
           <t>https://twitter.com/SFR</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -2502,24 +2712,34 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Electro Depot: chaine electromenager discount. Gros et petit electromenager, image, son, multimedia a prix bas.</t>
+          <t>Chaine de magasins electromenager discount. Concept depot pour reduire les couts. Gros et petit electromenager, image, son et multimedia a prix bas toute annee.</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
+          <t>Washing machines, fridges, ovens, dishwashers, TVs, audio, small appliances, multimedia</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Chain (80+ stores across France)</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
           <t>MDA</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>MDA (5), CE (3), SDA (2)</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr">
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -2581,24 +2801,34 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Cash Converters: achat et revente produits occasion. 62 magasins en France. Produits testes, garantis 1 an. Smartphones, PC, consoles, electromenager.</t>
+          <t>Leader mondial achat-revente aux particuliers. Present en France depuis 1994 avec 62 magasins. Produits occasion testes, expertises et garantis 1 an. Rayons hybrides: occasion, neuf et reconditionne.</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
+          <t>Smartphones, computers, tablets, video games, consoles, TVs, audio, small appliances, DVDs, books</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Chain / franchise (62 stores in France, 800+ worldwide in 23 countries)</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
           <t>Refurb</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>Refurb (5), CE (2)</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr">
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -2660,24 +2890,34 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
-          <t>PHOX: magasins photo specialises. Appareils photo, video, accessoires professionnels. Plus de 100 magasins en France depuis 1974.</t>
+          <t>Reseau de magasins photo specialises depuis 1974. Plus de 100 points de vente en France. Expert en appareils photo, video, accessoires professionnels. Services: labo photo, tirages, livres photo, studio.</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
+          <t>Cameras (reflex, hybrid, compact), lenses, video cameras, drones, tripods, camera bags, flashes, studio equipment, photo printing, photo books</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Buying group / franchise network (100+ independent photo stores under PHOX brand)</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
           <t>Photo</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>Photo (8)</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr">
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -2739,24 +2979,34 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Magasins BUT: meubles, electromenager, TV, Hi-Fi, multimedia. Plus de 330 magasins en France.</t>
+          <t>Enseigne francaise de meubles et electromenager. Plus de 330 magasins en France. Vend meubles, canapes, literie, decoration, electromenager, TV et Hi-Fi.</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
+          <t>Furniture, sofas, beds, decoration, washing machines, fridges, ovens, TVs, audio, small appliances</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Chain (330+ stores in France)</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
           <t>MDA</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>MDA (6), CE (3), SDA (2)</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr">
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -2818,24 +3068,34 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>LDLC: High-Tech Experience. Magasin informatique, reparation et depannage. Reseau de 100 magasins en France. PC, composants, peripheriques, multimedia.</t>
+          <t>Specialiste high-tech et informatique en ligne et en magasin. Reseau de 100 boutiques en France. Vente de PC, composants, peripheriques, gaming, multimedia. Offre aussi reparation et depannage.</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
+          <t>Computers, PC components, peripherals, monitors, printers, gaming, smartphones, tablets, networking, software</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Chain (100 franchise stores + e-commerce)</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
           <t>CE</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>CE (6)</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr">
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -2897,28 +3157,38 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
-          <t>LICK: boutique objets connectes, smartphones, tablettes, accessoires tendance. Reseau de magasins en France, partenaire Boulanger.</t>
+          <t>Boutique dediee aux objets connectes, smartphones, tablettes et accessoires tendance. Creee par le groupe Innov8 apres rachat de 17 boutiques The Phone House. Partenaire Boulanger.</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
+          <t>Smartphones, connected objects, tablets, phone cases, chargers, earbuds, speakers, smartwatches, connected home</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Chain (multiple stores in Paris, Bordeaux, Toulouse, Montpellier, Grenoble + e-commerce)</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
           <t>Phone Accessories</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>Phone Accessories (5), Mobile (3)</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>https://www.facebook.com/Lick.officiel</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr">
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -2935,7 +3205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2966,30 +3236,40 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>web_products</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>web_business_type</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>web_channel_guess</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>web_channel_detail</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>instagram</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>twitter</t>
         </is>
@@ -2998,306 +3278,386 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>302620747</t>
+          <t>353318981</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.but.fr</t>
+          <t>https://www.fnacdarty.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Magasins BUT: meubles, electromenager, TV, Hi-Fi, multimedia. Plus de 330 magasins en France.</t>
+          <t>Leader europeen de la distribution de produits electroniques, electromenager et biens culturels. Present dans 15 pays, 30000 employes, 1500 magasins. Groupe forme par le rachat de Darty par la Fnac en 2016.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MDA</t>
+          <t>Consumer electronics, household appliances, computers, TVs, audio, gaming, books, music, cultural goods</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>MDA (6), CE (3), SDA (2)</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+          <t>Chain (1500 stores in 15 countries)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>CE (5), MDA (3), SDA (2)</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fnac-darty</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>343744446</t>
+          <t>451355192</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.sfr.fr</t>
+          <t>https://www.boulanger.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1023</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>3011</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>contact@infos.boulanger.com</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SFR: operateur mobile et internet en France. Forfaits mobile, box internet, fibre.</t>
+          <t>Multi-specialiste electromenager et multimedia. Accompagne les clients dans le choix de produits techniques pour la maison et les loisirs, avec un accompagnement expert en magasin.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>TVs, audio, computers, tablets, phones, washing machines, fridges, ovens, dishwashers, small appliances, connected home</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Mobile (7)</t>
+          <t>Chain (130+ stores across France)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/SFR</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://twitter.com/SFR</t>
-        </is>
-      </c>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>CE (4), MDA (5), SDA (2)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/Boulanger.Electromenager.Multimedia</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>353318981</t>
+          <t>722023184</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.fnacdarty.com</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>https://www.orange.fr</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>3900</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>FNAC DARTY: leader europeen distribution electronique, electromenager, biens culturels. 1500 magasins, 30000 employes, present dans 15 pays.</t>
+          <t>Premier operateur telecom en France (classement ARCEP). Fournisseur de forfaits mobiles, internet fibre, TV. Boutiques physiques partout en France plus vente en ligne.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>Mobile phone plans, smartphones, fibre internet, TV packages, connected devices, phone accessories</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>CE (5), MDA (3), SDA (2)</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/fnac-darty</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr"/>
+          <t>Chain (1000+ stores in France, major telecom operator)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Mobile (8)</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/orange</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/orange</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>380129866</t>
+          <t>343744446</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.electrodepot.fr</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>https://www.sfr.fr</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1023</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Electro Depot: chaine electromenager discount. Gros et petit electromenager, image, son, multimedia a prix bas.</t>
+          <t>Deuxieme operateur telecom en France. Forfaits mobile, box internet fibre, TV. Reseau de boutiques SFR en France metropolitaine.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>MDA</t>
+          <t>Mobile phone plans, smartphones, fibre internet, TV packages, phone accessories</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>MDA (5), CE (3), SDA (2)</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
+          <t>Chain (500+ stores, major telecom operator)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Mobile (7)</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/SFR</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>https://twitter.com/SFR</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>440304385</t>
+          <t>380129866</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.ldlc.com</t>
+          <t>https://www.electrodepot.fr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>LDLC: High-Tech Experience. Magasin informatique, reparation et depannage. Reseau de 100 magasins en France. PC, composants, peripheriques, multimedia.</t>
+          <t>Chaine de magasins electromenager discount. Concept depot pour reduire les couts. Gros et petit electromenager, image, son et multimedia a prix bas toute annee.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>Washing machines, fridges, ovens, dishwashers, TVs, audio, small appliances, multimedia</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>CE (6)</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+          <t>Chain (80+ stores across France)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>MDA</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>MDA (5), CE (3), SDA (2)</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>451355192</t>
+          <t>302620747</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.boulanger.com</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>3011</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>contact@infos.boulanger.com</t>
-        </is>
-      </c>
+          <t>https://www.but.fr</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Boulanger: multi-specialiste electromenager et multimedia. Accompagne les clients dans amelioration du cadre de vie.</t>
+          <t>Enseigne francaise de meubles et electromenager. Plus de 330 magasins en France. Vend meubles, canapes, literie, decoration, electromenager, TV et Hi-Fi.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>Furniture, sofas, beds, decoration, washing machines, fridges, ovens, TVs, audio, small appliances</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>CE (4), MDA (5), SDA (2)</t>
+          <t>Chain (330+ stores in France)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/Boulanger.Electromenager.Multimedia</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
+          <t>MDA</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>MDA (6), CE (3), SDA (2)</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>503780322</t>
+          <t>440304385</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.phox.fr</t>
+          <t>https://www.ldlc.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>PHOX: magasins photo specialises. Appareils photo, video, accessoires professionnels. Plus de 100 magasins en France depuis 1974.</t>
+          <t>Specialiste high-tech et informatique en ligne et en magasin. Reseau de 100 boutiques en France. Vente de PC, composants, peripheriques, gaming, multimedia. Offre aussi reparation et depannage.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Photo</t>
+          <t>Computers, PC components, peripherals, monitors, printers, gaming, smartphones, tablets, networking, software</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Photo (8)</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+          <t>Chain (100 franchise stores + e-commerce)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>CE (6)</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>722023184</t>
+          <t>503780322</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.orange.fr</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>3900</t>
-        </is>
-      </c>
+          <t>https://www.phox.fr</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Orange: operateur telecom n1 en France. Mobile, internet fibre, TV. Boutiques partout en France.</t>
+          <t>Reseau de magasins photo specialises depuis 1974. Plus de 100 points de vente en France. Expert en appareils photo, video, accessoires professionnels. Services: labo photo, tirages, livres photo, studio.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Cameras (reflex, hybrid, compact), lenses, video cameras, drones, tripods, camera bags, flashes, studio equipment, photo printing, photo books</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Mobile (8)</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>Buying group / franchise network (100+ independent photo stores under PHOX brand)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/orange</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/orange</t>
-        </is>
-      </c>
+          <t>Photo (8)</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3314,23 +3674,33 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Cash Converters: achat et revente produits occasion. 62 magasins en France. Produits testes, garantis 1 an. Smartphones, PC, consoles, electromenager.</t>
+          <t>Leader mondial achat-revente aux particuliers. Present en France depuis 1994 avec 62 magasins. Produits occasion testes, expertises et garantis 1 an. Rayons hybrides: occasion, neuf et reconditionne.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>Smartphones, computers, tablets, video games, consoles, TVs, audio, small appliances, DVDs, books</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Chain / franchise (62 stores in France, 800+ worldwide in 23 countries)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>Refurb</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Refurb (5), CE (2)</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3347,27 +3717,37 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>LICK: boutique objets connectes, smartphones, tablettes, accessoires tendance. Reseau de magasins en France, partenaire Boulanger.</t>
+          <t>Boutique dediee aux objets connectes, smartphones, tablettes et accessoires tendance. Creee par le groupe Innov8 apres rachat de 17 boutiques The Phone House. Partenaire Boulanger.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>Smartphones, connected objects, tablets, phone cases, chargers, earbuds, speakers, smartwatches, connected home</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Chain (multiple stores in Paris, Bordeaux, Toulouse, Montpellier, Grenoble + e-commerce)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>Phone Accessories</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Phone Accessories (5), Mobile (3)</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>https://www.facebook.com/Lick.officiel</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>